<commit_message>
Docs: lote 6 de vitaminas con precios de oferta (solo imagen) y existencias al 13-oct
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VUzTHmv39QwMjbYWn5CWyp
</commit_message>
<xml_diff>
--- a/docs/marketing/LOTES-PUBLICIDAD-productos-y-precios.xlsx
+++ b/docs/marketing/LOTES-PUBLICIDAD-productos-y-precios.xlsx
@@ -12,7 +12,7 @@
     <sheet name="3 ISO (isolate)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4 Gainers" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5 Certificados (Klean y Muscle " sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6 Multivitaminicos y vitaminas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="6 Vitaminas OFERTA" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +33,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +48,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2A44"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,9 +68,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2347,32 +2359,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Precio RD$</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Precio normal RD$</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Precio de oferta RD$ (solo en la imagen)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Descuento %</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Existencia</t>
         </is>
@@ -2393,6 +2417,12 @@
         <v>1300</v>
       </c>
       <c r="D2" t="n">
+        <v>1105</v>
+      </c>
+      <c r="E2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2411,6 +2441,12 @@
         <v>1250</v>
       </c>
       <c r="D3" t="n">
+        <v>1063</v>
+      </c>
+      <c r="E3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F3" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2429,6 +2465,12 @@
         <v>1500</v>
       </c>
       <c r="D4" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F4" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2447,6 +2489,12 @@
         <v>1500</v>
       </c>
       <c r="D5" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2465,6 +2513,12 @@
         <v>1500</v>
       </c>
       <c r="D6" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2483,6 +2537,12 @@
         <v>1700</v>
       </c>
       <c r="D7" t="n">
+        <v>1445</v>
+      </c>
+      <c r="E7" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2501,7 +2561,13 @@
         <v>1450</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>856</v>
+      </c>
+      <c r="E8" t="n">
+        <v>41</v>
+      </c>
+      <c r="F8" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="9">
@@ -2519,6 +2585,12 @@
         <v>1600</v>
       </c>
       <c r="D9" t="n">
+        <v>1360</v>
+      </c>
+      <c r="E9" t="n">
+        <v>15</v>
+      </c>
+      <c r="F9" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2537,7 +2609,13 @@
         <v>1720</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>1462</v>
+      </c>
+      <c r="E10" t="n">
+        <v>15</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -2555,6 +2633,12 @@
         <v>2350</v>
       </c>
       <c r="D11" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E11" t="n">
+        <v>15</v>
+      </c>
+      <c r="F11" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2573,6 +2657,12 @@
         <v>1550</v>
       </c>
       <c r="D12" t="n">
+        <v>1318</v>
+      </c>
+      <c r="E12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2591,6 +2681,12 @@
         <v>1750</v>
       </c>
       <c r="D13" t="n">
+        <v>1488</v>
+      </c>
+      <c r="E13" t="n">
+        <v>15</v>
+      </c>
+      <c r="F13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2609,6 +2705,12 @@
         <v>1600</v>
       </c>
       <c r="D14" t="n">
+        <v>1360</v>
+      </c>
+      <c r="E14" t="n">
+        <v>15</v>
+      </c>
+      <c r="F14" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2627,6 +2729,12 @@
         <v>1700</v>
       </c>
       <c r="D15" t="n">
+        <v>1445</v>
+      </c>
+      <c r="E15" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2645,7 +2753,13 @@
         <v>1500</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>1275</v>
+      </c>
+      <c r="E16" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -2663,6 +2777,12 @@
         <v>1500</v>
       </c>
       <c r="D17" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2681,6 +2801,12 @@
         <v>1600</v>
       </c>
       <c r="D18" t="n">
+        <v>1360</v>
+      </c>
+      <c r="E18" t="n">
+        <v>15</v>
+      </c>
+      <c r="F18" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2699,6 +2825,12 @@
         <v>1500</v>
       </c>
       <c r="D19" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E19" t="n">
+        <v>15</v>
+      </c>
+      <c r="F19" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2717,6 +2849,12 @@
         <v>2450</v>
       </c>
       <c r="D20" t="n">
+        <v>2083</v>
+      </c>
+      <c r="E20" t="n">
+        <v>15</v>
+      </c>
+      <c r="F20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2735,6 +2873,12 @@
         <v>2900</v>
       </c>
       <c r="D21" t="n">
+        <v>2465</v>
+      </c>
+      <c r="E21" t="n">
+        <v>15</v>
+      </c>
+      <c r="F21" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2753,6 +2897,12 @@
         <v>1950</v>
       </c>
       <c r="D22" t="n">
+        <v>1658</v>
+      </c>
+      <c r="E22" t="n">
+        <v>15</v>
+      </c>
+      <c r="F22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2771,7 +2921,13 @@
         <v>2200</v>
       </c>
       <c r="D23" t="n">
-        <v>3</v>
+        <v>1870</v>
+      </c>
+      <c r="E23" t="n">
+        <v>15</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -2789,6 +2945,12 @@
         <v>1900</v>
       </c>
       <c r="D24" t="n">
+        <v>1615</v>
+      </c>
+      <c r="E24" t="n">
+        <v>15</v>
+      </c>
+      <c r="F24" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2807,6 +2969,12 @@
         <v>1500</v>
       </c>
       <c r="D25" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E25" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2825,6 +2993,12 @@
         <v>1500</v>
       </c>
       <c r="D26" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E26" t="n">
+        <v>15</v>
+      </c>
+      <c r="F26" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2843,6 +3017,12 @@
         <v>1500</v>
       </c>
       <c r="D27" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E27" t="n">
+        <v>15</v>
+      </c>
+      <c r="F27" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2861,6 +3041,12 @@
         <v>1400</v>
       </c>
       <c r="D28" t="n">
+        <v>1190</v>
+      </c>
+      <c r="E28" t="n">
+        <v>15</v>
+      </c>
+      <c r="F28" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2879,6 +3065,12 @@
         <v>1500</v>
       </c>
       <c r="D29" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E29" t="n">
+        <v>15</v>
+      </c>
+      <c r="F29" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2897,169 +3089,213 @@
         <v>2400</v>
       </c>
       <c r="D30" t="n">
+        <v>2040</v>
+      </c>
+      <c r="E30" t="n">
+        <v>15</v>
+      </c>
+      <c r="F30" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1055</t>
+          <t>1637</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Vitamin B-6 - Puritans Pride - 50 mg / 100 tabletas</t>
+          <t>Vitamin C - BioSteel</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1400</v>
+        <v>1500</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1275</v>
+      </c>
+      <c r="E31" t="n">
+        <v>15</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1637</t>
+          <t>1070</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Vitamin C - BioSteel</t>
+          <t>Vitamin D3 - Bronson Basics - 10,000 IU (250 mcg) / 360 unidades</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>1500</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>1275</v>
+      </c>
+      <c r="E32" t="n">
+        <v>15</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1070</t>
+          <t>1636</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Vitamin D3 - Bronson Basics - 10,000 IU (250 mcg) / 360 unidades</t>
+          <t>Vitamin E - Nature's Truth - 90 mg / 100 cápsulas</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>1500</v>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>1275</v>
+      </c>
+      <c r="E33" t="n">
+        <v>15</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1636</t>
+          <t>1051</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Vitamin E - Nature's Truth - 90 mg / 100 cápsulas</t>
+          <t>Vitamin E - Puritans Pride - 450 mg / 50 softgels</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>1500</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>1275</v>
+      </c>
+      <c r="E34" t="n">
+        <v>15</v>
+      </c>
+      <c r="F34" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1051</t>
+          <t>1052</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Vitamin E - Puritans Pride - 450 mg / 50 softgels</t>
+          <t>Vitamin K2+D3 - Bronson Basics - Envase blanco / 120 cápsulas</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1500</v>
+        <v>1750</v>
       </c>
       <c r="D35" t="n">
-        <v>2</v>
+        <v>1488</v>
+      </c>
+      <c r="E35" t="n">
+        <v>15</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1052</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Vitamin K2+D3 - Bronson Basics - Envase blanco / 120 cápsulas</t>
+          <t>Vitamin K2+D3 - Bronson Basics - Envase blanco / 60 cápsulas</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1750</v>
+        <v>1600</v>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>1360</v>
+      </c>
+      <c r="E36" t="n">
+        <v>15</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1211</t>
+          <t>1059</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Vitamin K2+D3 - Bronson Basics - Envase blanco / 60 cápsulas</t>
+          <t>Vitamin K2+D3 - Bronson Basics - Envase oscuro / 120 tabletas</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1600</v>
+        <v>1750</v>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>1488</v>
+      </c>
+      <c r="E37" t="n">
+        <v>15</v>
+      </c>
+      <c r="F37" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1059</t>
+          <t>1025</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Vitamin K2+D3 - Bronson Basics - Envase oscuro / 120 tabletas</t>
+          <t>Zinc Picolinate - Puritans Pride - 25 mg / 100 caplets</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1750</v>
+        <v>1500</v>
       </c>
       <c r="D38" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>1025</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Zinc Picolinate - Puritans Pride - 25 mg / 100 caplets</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D39" t="n">
+        <v>1275</v>
+      </c>
+      <c r="E38" t="n">
+        <v>15</v>
+      </c>
+      <c r="F38" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Vigencia: 12 al 31 de octubre de 2026. El precio de oferta NO se cambia en el sistema: la caja aplica el descuento en la factura. Margen mínimo 15 %.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>